<commit_message>
0.4.3 - Fixed bugs in Task Import.
</commit_message>
<xml_diff>
--- a/keel_trb_smart_template.xlsx
+++ b/keel_trb_smart_template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A068C57-7BE6-47F8-ADB3-6D12921EEBE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCA34F7D-6FF7-47E9-965A-4FCA6DAC8549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TRB Tasks" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="99">
   <si>
     <t>Function (Select from List)</t>
   </si>
@@ -187,13 +187,139 @@
   </si>
   <si>
     <t>A-VI/6</t>
+  </si>
+  <si>
+    <t>International Regulations for Preventing Collisions at Sea</t>
+  </si>
+  <si>
+    <t>COLREGS</t>
+  </si>
+  <si>
+    <t>Rule 01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learn and quote the COLREGS. Understand the legal implications and importance of each rule. </t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Rule 02</t>
+  </si>
+  <si>
+    <t>Rule 03</t>
+  </si>
+  <si>
+    <t>Rule 04</t>
+  </si>
+  <si>
+    <t>Rule 05</t>
+  </si>
+  <si>
+    <t>Rule 06</t>
+  </si>
+  <si>
+    <t>Rule 07</t>
+  </si>
+  <si>
+    <t>Rule 08</t>
+  </si>
+  <si>
+    <t>Rule 09</t>
+  </si>
+  <si>
+    <t>Rule 10</t>
+  </si>
+  <si>
+    <t>Rule 11</t>
+  </si>
+  <si>
+    <t>Rule 12</t>
+  </si>
+  <si>
+    <t>Rule 13</t>
+  </si>
+  <si>
+    <t>Rule 14</t>
+  </si>
+  <si>
+    <t>Rule 15</t>
+  </si>
+  <si>
+    <t>Rule 16</t>
+  </si>
+  <si>
+    <t>Rule 17</t>
+  </si>
+  <si>
+    <t>Rule 18</t>
+  </si>
+  <si>
+    <t>Rule 19</t>
+  </si>
+  <si>
+    <t>Rule 20</t>
+  </si>
+  <si>
+    <t>Rule 21</t>
+  </si>
+  <si>
+    <t>Rule 22</t>
+  </si>
+  <si>
+    <t>Rule 23</t>
+  </si>
+  <si>
+    <t>Rule 24</t>
+  </si>
+  <si>
+    <t>Rule 25</t>
+  </si>
+  <si>
+    <t>Rule 26</t>
+  </si>
+  <si>
+    <t>Rule 27</t>
+  </si>
+  <si>
+    <t>Rule 28</t>
+  </si>
+  <si>
+    <t>Rule 29</t>
+  </si>
+  <si>
+    <t>Rule 30</t>
+  </si>
+  <si>
+    <t>Rule 31</t>
+  </si>
+  <si>
+    <t>Rule 32</t>
+  </si>
+  <si>
+    <t>Rule 33</t>
+  </si>
+  <si>
+    <t>Rule 34</t>
+  </si>
+  <si>
+    <t>Rule 35</t>
+  </si>
+  <si>
+    <t>Rule 36</t>
+  </si>
+  <si>
+    <t>Rule 37</t>
+  </si>
+  <si>
+    <t>Rule 38</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,6 +332,12 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -575,7 +707,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -632,7 +764,1566 @@
         <v>12</v>
       </c>
     </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s">
+        <v>61</v>
+      </c>
+      <c r="J3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="s">
+        <v>18</v>
+      </c>
+      <c r="M3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" t="s">
+        <v>61</v>
+      </c>
+      <c r="J4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="s">
+        <v>18</v>
+      </c>
+      <c r="M4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>61</v>
+      </c>
+      <c r="J5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" t="s">
+        <v>61</v>
+      </c>
+      <c r="J6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" t="s">
+        <v>61</v>
+      </c>
+      <c r="J7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="s">
+        <v>18</v>
+      </c>
+      <c r="M7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J8" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="s">
+        <v>18</v>
+      </c>
+      <c r="M8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" t="s">
+        <v>68</v>
+      </c>
+      <c r="E9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" t="s">
+        <v>61</v>
+      </c>
+      <c r="J9" t="s">
+        <v>24</v>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="s">
+        <v>18</v>
+      </c>
+      <c r="M9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" t="s">
+        <v>69</v>
+      </c>
+      <c r="E10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" t="s">
+        <v>61</v>
+      </c>
+      <c r="J10" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="s">
+        <v>18</v>
+      </c>
+      <c r="M10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" t="s">
+        <v>61</v>
+      </c>
+      <c r="J11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="s">
+        <v>18</v>
+      </c>
+      <c r="M11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" t="s">
+        <v>61</v>
+      </c>
+      <c r="J12" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" t="s">
+        <v>18</v>
+      </c>
+      <c r="M12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" t="s">
+        <v>61</v>
+      </c>
+      <c r="J13" t="s">
+        <v>24</v>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" t="s">
+        <v>18</v>
+      </c>
+      <c r="M13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" t="s">
+        <v>61</v>
+      </c>
+      <c r="J14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" t="s">
+        <v>18</v>
+      </c>
+      <c r="M14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" t="s">
+        <v>61</v>
+      </c>
+      <c r="J15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" t="s">
+        <v>18</v>
+      </c>
+      <c r="M15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" t="s">
+        <v>60</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" t="s">
+        <v>61</v>
+      </c>
+      <c r="J16" t="s">
+        <v>24</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" t="s">
+        <v>18</v>
+      </c>
+      <c r="M16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J17" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" t="s">
+        <v>18</v>
+      </c>
+      <c r="M17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" t="s">
+        <v>61</v>
+      </c>
+      <c r="J18" t="s">
+        <v>24</v>
+      </c>
+      <c r="K18" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" t="s">
+        <v>18</v>
+      </c>
+      <c r="M18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" t="s">
+        <v>61</v>
+      </c>
+      <c r="J19" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" t="s">
+        <v>18</v>
+      </c>
+      <c r="M19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" t="s">
+        <v>61</v>
+      </c>
+      <c r="J20" t="s">
+        <v>24</v>
+      </c>
+      <c r="K20" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" t="s">
+        <v>18</v>
+      </c>
+      <c r="M20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" t="s">
+        <v>80</v>
+      </c>
+      <c r="E21" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" t="s">
+        <v>61</v>
+      </c>
+      <c r="J21" t="s">
+        <v>24</v>
+      </c>
+      <c r="K21" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" t="s">
+        <v>18</v>
+      </c>
+      <c r="M21" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="s">
+        <v>16</v>
+      </c>
+      <c r="I22" t="s">
+        <v>61</v>
+      </c>
+      <c r="J22" t="s">
+        <v>24</v>
+      </c>
+      <c r="K22" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" t="s">
+        <v>18</v>
+      </c>
+      <c r="M22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" t="s">
+        <v>82</v>
+      </c>
+      <c r="E23" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" t="s">
+        <v>61</v>
+      </c>
+      <c r="J23" t="s">
+        <v>24</v>
+      </c>
+      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" t="s">
+        <v>18</v>
+      </c>
+      <c r="M23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" t="s">
+        <v>61</v>
+      </c>
+      <c r="J24" t="s">
+        <v>24</v>
+      </c>
+      <c r="K24" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" t="s">
+        <v>18</v>
+      </c>
+      <c r="M24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" t="s">
+        <v>58</v>
+      </c>
+      <c r="D25" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" t="s">
+        <v>60</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" t="s">
+        <v>61</v>
+      </c>
+      <c r="J25" t="s">
+        <v>24</v>
+      </c>
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" t="s">
+        <v>18</v>
+      </c>
+      <c r="M25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" t="s">
+        <v>85</v>
+      </c>
+      <c r="E26" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" t="s">
+        <v>61</v>
+      </c>
+      <c r="J26" t="s">
+        <v>24</v>
+      </c>
+      <c r="K26" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" t="s">
+        <v>18</v>
+      </c>
+      <c r="M26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" t="s">
+        <v>58</v>
+      </c>
+      <c r="D27" t="s">
+        <v>86</v>
+      </c>
+      <c r="E27" t="s">
+        <v>60</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" t="s">
+        <v>61</v>
+      </c>
+      <c r="J27" t="s">
+        <v>24</v>
+      </c>
+      <c r="K27" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" t="s">
+        <v>18</v>
+      </c>
+      <c r="M27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" t="s">
+        <v>87</v>
+      </c>
+      <c r="E28" t="s">
+        <v>60</v>
+      </c>
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" t="s">
+        <v>61</v>
+      </c>
+      <c r="J28" t="s">
+        <v>24</v>
+      </c>
+      <c r="K28" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" t="s">
+        <v>18</v>
+      </c>
+      <c r="M28" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" t="s">
+        <v>88</v>
+      </c>
+      <c r="E29" t="s">
+        <v>60</v>
+      </c>
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" t="s">
+        <v>16</v>
+      </c>
+      <c r="I29" t="s">
+        <v>61</v>
+      </c>
+      <c r="J29" t="s">
+        <v>24</v>
+      </c>
+      <c r="K29" t="b">
+        <v>1</v>
+      </c>
+      <c r="L29" t="s">
+        <v>18</v>
+      </c>
+      <c r="M29" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" t="s">
+        <v>58</v>
+      </c>
+      <c r="D30" t="s">
+        <v>89</v>
+      </c>
+      <c r="E30" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" t="s">
+        <v>61</v>
+      </c>
+      <c r="J30" t="s">
+        <v>24</v>
+      </c>
+      <c r="K30" t="b">
+        <v>1</v>
+      </c>
+      <c r="L30" t="s">
+        <v>18</v>
+      </c>
+      <c r="M30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" t="s">
+        <v>60</v>
+      </c>
+      <c r="F31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" t="s">
+        <v>61</v>
+      </c>
+      <c r="J31" t="s">
+        <v>24</v>
+      </c>
+      <c r="K31" t="b">
+        <v>1</v>
+      </c>
+      <c r="L31" t="s">
+        <v>18</v>
+      </c>
+      <c r="M31" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>13</v>
+      </c>
+      <c r="B32" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" t="s">
+        <v>58</v>
+      </c>
+      <c r="D32" t="s">
+        <v>91</v>
+      </c>
+      <c r="E32" t="s">
+        <v>60</v>
+      </c>
+      <c r="F32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="s">
+        <v>16</v>
+      </c>
+      <c r="I32" t="s">
+        <v>61</v>
+      </c>
+      <c r="J32" t="s">
+        <v>24</v>
+      </c>
+      <c r="K32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L32" t="s">
+        <v>18</v>
+      </c>
+      <c r="M32" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33" t="s">
+        <v>58</v>
+      </c>
+      <c r="D33" t="s">
+        <v>92</v>
+      </c>
+      <c r="E33" t="s">
+        <v>60</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" t="s">
+        <v>61</v>
+      </c>
+      <c r="J33" t="s">
+        <v>24</v>
+      </c>
+      <c r="K33" t="b">
+        <v>1</v>
+      </c>
+      <c r="L33" t="s">
+        <v>18</v>
+      </c>
+      <c r="M33" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" t="s">
+        <v>93</v>
+      </c>
+      <c r="E34" t="s">
+        <v>60</v>
+      </c>
+      <c r="F34" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" t="s">
+        <v>61</v>
+      </c>
+      <c r="J34" t="s">
+        <v>24</v>
+      </c>
+      <c r="K34" t="b">
+        <v>1</v>
+      </c>
+      <c r="L34" t="s">
+        <v>18</v>
+      </c>
+      <c r="M34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" t="s">
+        <v>58</v>
+      </c>
+      <c r="D35" t="s">
+        <v>94</v>
+      </c>
+      <c r="E35" t="s">
+        <v>60</v>
+      </c>
+      <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" t="s">
+        <v>61</v>
+      </c>
+      <c r="J35" t="s">
+        <v>24</v>
+      </c>
+      <c r="K35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L35" t="s">
+        <v>18</v>
+      </c>
+      <c r="M35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" t="s">
+        <v>58</v>
+      </c>
+      <c r="D36" t="s">
+        <v>95</v>
+      </c>
+      <c r="E36" t="s">
+        <v>60</v>
+      </c>
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" t="s">
+        <v>16</v>
+      </c>
+      <c r="I36" t="s">
+        <v>61</v>
+      </c>
+      <c r="J36" t="s">
+        <v>24</v>
+      </c>
+      <c r="K36" t="b">
+        <v>1</v>
+      </c>
+      <c r="L36" t="s">
+        <v>18</v>
+      </c>
+      <c r="M36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" t="s">
+        <v>58</v>
+      </c>
+      <c r="D37" t="s">
+        <v>96</v>
+      </c>
+      <c r="E37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F37" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" t="s">
+        <v>16</v>
+      </c>
+      <c r="I37" t="s">
+        <v>61</v>
+      </c>
+      <c r="J37" t="s">
+        <v>24</v>
+      </c>
+      <c r="K37" t="b">
+        <v>1</v>
+      </c>
+      <c r="L37" t="s">
+        <v>18</v>
+      </c>
+      <c r="M37" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" t="s">
+        <v>58</v>
+      </c>
+      <c r="D38" t="s">
+        <v>97</v>
+      </c>
+      <c r="E38" t="s">
+        <v>60</v>
+      </c>
+      <c r="F38" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I38" t="s">
+        <v>61</v>
+      </c>
+      <c r="J38" t="s">
+        <v>24</v>
+      </c>
+      <c r="K38" t="b">
+        <v>1</v>
+      </c>
+      <c r="L38" t="s">
+        <v>18</v>
+      </c>
+      <c r="M38" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39" t="s">
+        <v>58</v>
+      </c>
+      <c r="D39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E39" t="s">
+        <v>60</v>
+      </c>
+      <c r="F39" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39" t="s">
+        <v>61</v>
+      </c>
+      <c r="J39" t="s">
+        <v>24</v>
+      </c>
+      <c r="K39" t="b">
+        <v>1</v>
+      </c>
+      <c r="L39" t="s">
+        <v>18</v>
+      </c>
+      <c r="M39" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="K2:K500" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"TRUE,FALSE"</formula1>

</xml_diff>

<commit_message>
0.5.1 - Working on routes.
</commit_message>
<xml_diff>
--- a/keel_trb_smart_template.xlsx
+++ b/keel_trb_smart_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCA34F7D-6FF7-47E9-965A-4FCA6DAC8549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F695D5D-BFA6-47D9-8F5F-B1E3ECE9519A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="141">
   <si>
     <t>Function (Select from List)</t>
   </si>
@@ -313,6 +313,132 @@
   </si>
   <si>
     <t>Rule 38</t>
+  </si>
+  <si>
+    <t>Plan and conduct a passage and determine position</t>
+  </si>
+  <si>
+    <t>Consult Navigational publications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demonstrate an understanding of the chart folio system and assist in correcting charts and other publications. </t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of contents and the use of Notices to mariners</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of contents and the use of Sailing directions and ship's routeing information</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of contents and the use of List of lights and fog signals</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of contents and the use of Tide tables, tidal stream and current atlases</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of contents and the use of Pilot books</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of contents and the use of Radio navigational warnings</t>
+  </si>
+  <si>
+    <t>Select charts of adequate scale</t>
+  </si>
+  <si>
+    <t>Assist deck officer in preparing navigational passages and in voyage planning</t>
+  </si>
+  <si>
+    <t>Select appropriate scale chart from paper chart portfolio, Electronic Chart System (ECSJ or Electronic Chart Display and Information Systems (ECDIS)</t>
+  </si>
+  <si>
+    <t>Set up Course Recorder</t>
+  </si>
+  <si>
+    <t>Set up Off course alarm</t>
+  </si>
+  <si>
+    <t>Calculate Estimated Time of Arrival (ETA)</t>
+  </si>
+  <si>
+    <t>Practise tidal calculations</t>
+  </si>
+  <si>
+    <t>Practise calculat ions for distance, average speed, course made good, set and drift, ETA</t>
+  </si>
+  <si>
+    <t>Determine and apply compass error for courses and compass bearings</t>
+  </si>
+  <si>
+    <t>Apply magnetic variation and deviation</t>
+  </si>
+  <si>
+    <t>Practise use of the azimuth mirror</t>
+  </si>
+  <si>
+    <t>Practice Azimuths</t>
+  </si>
+  <si>
+    <t>Practice Amplitudes</t>
+  </si>
+  <si>
+    <t>Understand the use of and make ent ries in the compass error book and interpre.t information recorded</t>
+  </si>
+  <si>
+    <t>Demonstrate the use of the compass when setting course</t>
+  </si>
+  <si>
+    <t>Estimate and make allowance for leeway and tidal currents</t>
+  </si>
+  <si>
+    <t>Set Courses</t>
+  </si>
+  <si>
+    <t>Recognise conspicusous objects and other terrestrial/celestial aids to navigation in daylight and at night</t>
+  </si>
+  <si>
+    <t>Perform look-out duties and report objects in degrees or points</t>
+  </si>
+  <si>
+    <t>Identify aids to navigation including lighthouses, beacons and buoys</t>
+  </si>
+  <si>
+    <t>Identify star constellations and stars of first magnitude and learn to use star chart and star finder</t>
+  </si>
+  <si>
+    <t>Practice compass bearings and visual fixes</t>
+  </si>
+  <si>
+    <t>Demostrate a knowledge of the IALA system of buoyage</t>
+  </si>
+  <si>
+    <t>Use azimuth mirror and sextant to fix ship's position by celestial and terrestrial observations</t>
+  </si>
+  <si>
+    <t>Use azimuth mirror to fix ship's position</t>
+  </si>
+  <si>
+    <t>Use a sextant and demonstrate how to identify and remove errors</t>
+  </si>
+  <si>
+    <t>Practice horizontal and vertical sextant angles</t>
+  </si>
+  <si>
+    <t>Make noon calculations e.g. distance, average speed, course made good, set and drift and ETA</t>
+  </si>
+  <si>
+    <t>State ship's position by dead reckoning</t>
+  </si>
+  <si>
+    <t>Operate all electronic navigational equipment to ascertain the ship's position</t>
+  </si>
+  <si>
+    <t>Practice Radar switch on and set up procedure</t>
+  </si>
+  <si>
+    <t>Practice Radar Plotting</t>
+  </si>
+  <si>
+    <t>Practice Position fixes by radar</t>
   </si>
 </sst>
 </file>
@@ -365,9 +491,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -2320,6 +2447,1336 @@
       </c>
       <c r="M39" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" t="s">
+        <v>100</v>
+      </c>
+      <c r="D40" t="s">
+        <v>101</v>
+      </c>
+      <c r="F40" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" t="s">
+        <v>16</v>
+      </c>
+      <c r="I40" t="s">
+        <v>61</v>
+      </c>
+      <c r="J40" t="s">
+        <v>24</v>
+      </c>
+      <c r="K40" t="b">
+        <v>1</v>
+      </c>
+      <c r="L40" t="s">
+        <v>25</v>
+      </c>
+      <c r="M40" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" t="s">
+        <v>99</v>
+      </c>
+      <c r="C41" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41" t="s">
+        <v>102</v>
+      </c>
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" t="s">
+        <v>61</v>
+      </c>
+      <c r="J41" t="s">
+        <v>24</v>
+      </c>
+      <c r="K41" t="b">
+        <v>1</v>
+      </c>
+      <c r="L41" t="s">
+        <v>25</v>
+      </c>
+      <c r="M41" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42" t="s">
+        <v>99</v>
+      </c>
+      <c r="C42" t="s">
+        <v>100</v>
+      </c>
+      <c r="D42" t="s">
+        <v>103</v>
+      </c>
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" t="s">
+        <v>16</v>
+      </c>
+      <c r="I42" t="s">
+        <v>61</v>
+      </c>
+      <c r="J42" t="s">
+        <v>24</v>
+      </c>
+      <c r="K42" t="b">
+        <v>1</v>
+      </c>
+      <c r="L42" t="s">
+        <v>25</v>
+      </c>
+      <c r="M42" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43" t="s">
+        <v>99</v>
+      </c>
+      <c r="C43" t="s">
+        <v>100</v>
+      </c>
+      <c r="D43" t="s">
+        <v>104</v>
+      </c>
+      <c r="F43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" t="s">
+        <v>61</v>
+      </c>
+      <c r="J43" t="s">
+        <v>24</v>
+      </c>
+      <c r="K43" t="b">
+        <v>1</v>
+      </c>
+      <c r="L43" t="s">
+        <v>25</v>
+      </c>
+      <c r="M43" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" t="s">
+        <v>100</v>
+      </c>
+      <c r="D44" t="s">
+        <v>105</v>
+      </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" t="s">
+        <v>61</v>
+      </c>
+      <c r="J44" t="s">
+        <v>24</v>
+      </c>
+      <c r="K44" t="b">
+        <v>1</v>
+      </c>
+      <c r="L44" t="s">
+        <v>25</v>
+      </c>
+      <c r="M44" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" t="s">
+        <v>99</v>
+      </c>
+      <c r="C45" t="s">
+        <v>100</v>
+      </c>
+      <c r="D45" t="s">
+        <v>106</v>
+      </c>
+      <c r="F45" t="s">
+        <v>14</v>
+      </c>
+      <c r="G45" t="s">
+        <v>15</v>
+      </c>
+      <c r="H45" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" t="s">
+        <v>61</v>
+      </c>
+      <c r="J45" t="s">
+        <v>24</v>
+      </c>
+      <c r="K45" t="b">
+        <v>1</v>
+      </c>
+      <c r="L45" t="s">
+        <v>25</v>
+      </c>
+      <c r="M45" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>13</v>
+      </c>
+      <c r="B46" t="s">
+        <v>99</v>
+      </c>
+      <c r="C46" t="s">
+        <v>100</v>
+      </c>
+      <c r="D46" t="s">
+        <v>107</v>
+      </c>
+      <c r="F46" t="s">
+        <v>14</v>
+      </c>
+      <c r="G46" t="s">
+        <v>15</v>
+      </c>
+      <c r="H46" t="s">
+        <v>16</v>
+      </c>
+      <c r="I46" t="s">
+        <v>61</v>
+      </c>
+      <c r="J46" t="s">
+        <v>24</v>
+      </c>
+      <c r="K46" t="b">
+        <v>1</v>
+      </c>
+      <c r="L46" t="s">
+        <v>25</v>
+      </c>
+      <c r="M46" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" t="s">
+        <v>99</v>
+      </c>
+      <c r="C47" t="s">
+        <v>108</v>
+      </c>
+      <c r="D47" t="s">
+        <v>109</v>
+      </c>
+      <c r="F47" t="s">
+        <v>14</v>
+      </c>
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" t="s">
+        <v>61</v>
+      </c>
+      <c r="J47" t="s">
+        <v>24</v>
+      </c>
+      <c r="K47" t="b">
+        <v>1</v>
+      </c>
+      <c r="L47" t="s">
+        <v>18</v>
+      </c>
+      <c r="M47" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" t="s">
+        <v>108</v>
+      </c>
+      <c r="D48" t="s">
+        <v>110</v>
+      </c>
+      <c r="F48" t="s">
+        <v>14</v>
+      </c>
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" t="s">
+        <v>61</v>
+      </c>
+      <c r="J48" t="s">
+        <v>24</v>
+      </c>
+      <c r="K48" t="b">
+        <v>1</v>
+      </c>
+      <c r="L48" t="s">
+        <v>18</v>
+      </c>
+      <c r="M48" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49" t="s">
+        <v>99</v>
+      </c>
+      <c r="C49" t="s">
+        <v>124</v>
+      </c>
+      <c r="D49" t="s">
+        <v>122</v>
+      </c>
+      <c r="F49" t="s">
+        <v>14</v>
+      </c>
+      <c r="G49" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" t="s">
+        <v>61</v>
+      </c>
+      <c r="J49" t="s">
+        <v>24</v>
+      </c>
+      <c r="K49" t="b">
+        <v>1</v>
+      </c>
+      <c r="L49" t="s">
+        <v>18</v>
+      </c>
+      <c r="M49" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>13</v>
+      </c>
+      <c r="B50" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" t="s">
+        <v>124</v>
+      </c>
+      <c r="D50" t="s">
+        <v>111</v>
+      </c>
+      <c r="F50" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" t="s">
+        <v>16</v>
+      </c>
+      <c r="I50" t="s">
+        <v>61</v>
+      </c>
+      <c r="J50" t="s">
+        <v>24</v>
+      </c>
+      <c r="K50" t="b">
+        <v>1</v>
+      </c>
+      <c r="L50" t="s">
+        <v>18</v>
+      </c>
+      <c r="M50" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>13</v>
+      </c>
+      <c r="B51" t="s">
+        <v>99</v>
+      </c>
+      <c r="C51" t="s">
+        <v>124</v>
+      </c>
+      <c r="D51" t="s">
+        <v>112</v>
+      </c>
+      <c r="F51" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" t="s">
+        <v>16</v>
+      </c>
+      <c r="I51" t="s">
+        <v>61</v>
+      </c>
+      <c r="J51" t="s">
+        <v>24</v>
+      </c>
+      <c r="K51" t="b">
+        <v>1</v>
+      </c>
+      <c r="L51" t="s">
+        <v>18</v>
+      </c>
+      <c r="M51" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>13</v>
+      </c>
+      <c r="B52" t="s">
+        <v>99</v>
+      </c>
+      <c r="C52" t="s">
+        <v>124</v>
+      </c>
+      <c r="D52" t="s">
+        <v>123</v>
+      </c>
+      <c r="F52" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" t="s">
+        <v>16</v>
+      </c>
+      <c r="I52" t="s">
+        <v>61</v>
+      </c>
+      <c r="J52" t="s">
+        <v>24</v>
+      </c>
+      <c r="K52" t="b">
+        <v>1</v>
+      </c>
+      <c r="L52" t="s">
+        <v>18</v>
+      </c>
+      <c r="M52" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>13</v>
+      </c>
+      <c r="B53" t="s">
+        <v>99</v>
+      </c>
+      <c r="C53" t="s">
+        <v>124</v>
+      </c>
+      <c r="D53" t="s">
+        <v>114</v>
+      </c>
+      <c r="F53" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" t="s">
+        <v>15</v>
+      </c>
+      <c r="H53" t="s">
+        <v>16</v>
+      </c>
+      <c r="I53" t="s">
+        <v>61</v>
+      </c>
+      <c r="J53" t="s">
+        <v>24</v>
+      </c>
+      <c r="K53" t="b">
+        <v>1</v>
+      </c>
+      <c r="L53" t="s">
+        <v>18</v>
+      </c>
+      <c r="M53" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>13</v>
+      </c>
+      <c r="B54" t="s">
+        <v>99</v>
+      </c>
+      <c r="C54" t="s">
+        <v>113</v>
+      </c>
+      <c r="D54" t="s">
+        <v>115</v>
+      </c>
+      <c r="F54" t="s">
+        <v>14</v>
+      </c>
+      <c r="G54" t="s">
+        <v>15</v>
+      </c>
+      <c r="H54" t="s">
+        <v>16</v>
+      </c>
+      <c r="I54" t="s">
+        <v>61</v>
+      </c>
+      <c r="J54" t="s">
+        <v>24</v>
+      </c>
+      <c r="K54" t="b">
+        <v>1</v>
+      </c>
+      <c r="L54" t="s">
+        <v>18</v>
+      </c>
+      <c r="M54" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>13</v>
+      </c>
+      <c r="B55" t="s">
+        <v>99</v>
+      </c>
+      <c r="C55" t="s">
+        <v>116</v>
+      </c>
+      <c r="D55" t="s">
+        <v>117</v>
+      </c>
+      <c r="F55" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" t="s">
+        <v>16</v>
+      </c>
+      <c r="I55" t="s">
+        <v>61</v>
+      </c>
+      <c r="J55" t="s">
+        <v>24</v>
+      </c>
+      <c r="K55" t="b">
+        <v>1</v>
+      </c>
+      <c r="L55" t="s">
+        <v>18</v>
+      </c>
+      <c r="M55" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>13</v>
+      </c>
+      <c r="B56" t="s">
+        <v>99</v>
+      </c>
+      <c r="C56" t="s">
+        <v>116</v>
+      </c>
+      <c r="D56" t="s">
+        <v>118</v>
+      </c>
+      <c r="F56" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" t="s">
+        <v>16</v>
+      </c>
+      <c r="I56" t="s">
+        <v>61</v>
+      </c>
+      <c r="J56" t="s">
+        <v>24</v>
+      </c>
+      <c r="K56" t="b">
+        <v>1</v>
+      </c>
+      <c r="L56" t="s">
+        <v>18</v>
+      </c>
+      <c r="M56" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>13</v>
+      </c>
+      <c r="B57" t="s">
+        <v>99</v>
+      </c>
+      <c r="C57" t="s">
+        <v>116</v>
+      </c>
+      <c r="D57" t="s">
+        <v>119</v>
+      </c>
+      <c r="F57" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" t="s">
+        <v>16</v>
+      </c>
+      <c r="I57" t="s">
+        <v>61</v>
+      </c>
+      <c r="J57" t="s">
+        <v>24</v>
+      </c>
+      <c r="K57" t="b">
+        <v>1</v>
+      </c>
+      <c r="L57" t="s">
+        <v>18</v>
+      </c>
+      <c r="M57" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>13</v>
+      </c>
+      <c r="B58" t="s">
+        <v>99</v>
+      </c>
+      <c r="C58" t="s">
+        <v>116</v>
+      </c>
+      <c r="D58" t="s">
+        <v>120</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58" t="s">
+        <v>15</v>
+      </c>
+      <c r="H58" t="s">
+        <v>16</v>
+      </c>
+      <c r="I58" t="s">
+        <v>61</v>
+      </c>
+      <c r="J58" t="s">
+        <v>24</v>
+      </c>
+      <c r="K58" t="b">
+        <v>1</v>
+      </c>
+      <c r="L58" t="s">
+        <v>18</v>
+      </c>
+      <c r="M58" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>13</v>
+      </c>
+      <c r="B59" t="s">
+        <v>99</v>
+      </c>
+      <c r="C59" t="s">
+        <v>116</v>
+      </c>
+      <c r="D59" t="s">
+        <v>121</v>
+      </c>
+      <c r="F59" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59" t="s">
+        <v>15</v>
+      </c>
+      <c r="H59" t="s">
+        <v>16</v>
+      </c>
+      <c r="I59" t="s">
+        <v>61</v>
+      </c>
+      <c r="J59" t="s">
+        <v>24</v>
+      </c>
+      <c r="K59" t="b">
+        <v>1</v>
+      </c>
+      <c r="L59" t="s">
+        <v>18</v>
+      </c>
+      <c r="M59" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60" t="s">
+        <v>99</v>
+      </c>
+      <c r="C60" t="s">
+        <v>125</v>
+      </c>
+      <c r="D60" t="s">
+        <v>126</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60" t="s">
+        <v>15</v>
+      </c>
+      <c r="H60" t="s">
+        <v>16</v>
+      </c>
+      <c r="I60" t="s">
+        <v>61</v>
+      </c>
+      <c r="J60" t="s">
+        <v>24</v>
+      </c>
+      <c r="K60" t="b">
+        <v>1</v>
+      </c>
+      <c r="L60" t="s">
+        <v>18</v>
+      </c>
+      <c r="M60" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61" t="s">
+        <v>99</v>
+      </c>
+      <c r="C61" t="s">
+        <v>125</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F61" t="s">
+        <v>14</v>
+      </c>
+      <c r="G61" t="s">
+        <v>15</v>
+      </c>
+      <c r="H61" t="s">
+        <v>16</v>
+      </c>
+      <c r="I61" t="s">
+        <v>61</v>
+      </c>
+      <c r="J61" t="s">
+        <v>24</v>
+      </c>
+      <c r="K61" t="b">
+        <v>1</v>
+      </c>
+      <c r="L61" t="s">
+        <v>18</v>
+      </c>
+      <c r="M61" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>13</v>
+      </c>
+      <c r="B62" t="s">
+        <v>99</v>
+      </c>
+      <c r="C62" t="s">
+        <v>125</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F62" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62" t="s">
+        <v>15</v>
+      </c>
+      <c r="H62" t="s">
+        <v>16</v>
+      </c>
+      <c r="I62" t="s">
+        <v>61</v>
+      </c>
+      <c r="J62" t="s">
+        <v>24</v>
+      </c>
+      <c r="K62" t="b">
+        <v>1</v>
+      </c>
+      <c r="L62" t="s">
+        <v>18</v>
+      </c>
+      <c r="M62" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>13</v>
+      </c>
+      <c r="B63" t="s">
+        <v>99</v>
+      </c>
+      <c r="C63" t="s">
+        <v>125</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F63" t="s">
+        <v>14</v>
+      </c>
+      <c r="G63" t="s">
+        <v>15</v>
+      </c>
+      <c r="H63" t="s">
+        <v>16</v>
+      </c>
+      <c r="I63" t="s">
+        <v>61</v>
+      </c>
+      <c r="J63" t="s">
+        <v>24</v>
+      </c>
+      <c r="K63" t="b">
+        <v>1</v>
+      </c>
+      <c r="L63" t="s">
+        <v>18</v>
+      </c>
+      <c r="M63" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>13</v>
+      </c>
+      <c r="B64" t="s">
+        <v>99</v>
+      </c>
+      <c r="C64" t="s">
+        <v>125</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F64" t="s">
+        <v>14</v>
+      </c>
+      <c r="G64" t="s">
+        <v>15</v>
+      </c>
+      <c r="H64" t="s">
+        <v>16</v>
+      </c>
+      <c r="I64" t="s">
+        <v>61</v>
+      </c>
+      <c r="J64" t="s">
+        <v>24</v>
+      </c>
+      <c r="K64" t="b">
+        <v>1</v>
+      </c>
+      <c r="L64" t="s">
+        <v>18</v>
+      </c>
+      <c r="M64" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>13</v>
+      </c>
+      <c r="B65" t="s">
+        <v>99</v>
+      </c>
+      <c r="C65" t="s">
+        <v>131</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F65" t="s">
+        <v>14</v>
+      </c>
+      <c r="G65" t="s">
+        <v>15</v>
+      </c>
+      <c r="H65" t="s">
+        <v>16</v>
+      </c>
+      <c r="I65" t="s">
+        <v>61</v>
+      </c>
+      <c r="J65" t="s">
+        <v>24</v>
+      </c>
+      <c r="K65" t="b">
+        <v>1</v>
+      </c>
+      <c r="L65" t="s">
+        <v>18</v>
+      </c>
+      <c r="M65" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>13</v>
+      </c>
+      <c r="B66" t="s">
+        <v>99</v>
+      </c>
+      <c r="C66" t="s">
+        <v>131</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F66" t="s">
+        <v>14</v>
+      </c>
+      <c r="G66" t="s">
+        <v>15</v>
+      </c>
+      <c r="H66" t="s">
+        <v>16</v>
+      </c>
+      <c r="I66" t="s">
+        <v>61</v>
+      </c>
+      <c r="J66" t="s">
+        <v>24</v>
+      </c>
+      <c r="K66" t="b">
+        <v>1</v>
+      </c>
+      <c r="L66" t="s">
+        <v>18</v>
+      </c>
+      <c r="M66" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>13</v>
+      </c>
+      <c r="B67" t="s">
+        <v>99</v>
+      </c>
+      <c r="C67" t="s">
+        <v>131</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F67" t="s">
+        <v>14</v>
+      </c>
+      <c r="G67" t="s">
+        <v>15</v>
+      </c>
+      <c r="H67" t="s">
+        <v>16</v>
+      </c>
+      <c r="I67" t="s">
+        <v>61</v>
+      </c>
+      <c r="J67" t="s">
+        <v>24</v>
+      </c>
+      <c r="K67" t="b">
+        <v>1</v>
+      </c>
+      <c r="L67" t="s">
+        <v>18</v>
+      </c>
+      <c r="M67" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>13</v>
+      </c>
+      <c r="B68" t="s">
+        <v>99</v>
+      </c>
+      <c r="C68" t="s">
+        <v>131</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F68" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68" t="s">
+        <v>15</v>
+      </c>
+      <c r="H68" t="s">
+        <v>16</v>
+      </c>
+      <c r="I68" t="s">
+        <v>61</v>
+      </c>
+      <c r="J68" t="s">
+        <v>24</v>
+      </c>
+      <c r="K68" t="b">
+        <v>1</v>
+      </c>
+      <c r="L68" t="s">
+        <v>18</v>
+      </c>
+      <c r="M68" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>13</v>
+      </c>
+      <c r="B69" t="s">
+        <v>99</v>
+      </c>
+      <c r="C69" t="s">
+        <v>136</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F69" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" t="s">
+        <v>15</v>
+      </c>
+      <c r="H69" t="s">
+        <v>16</v>
+      </c>
+      <c r="I69" t="s">
+        <v>61</v>
+      </c>
+      <c r="J69" t="s">
+        <v>24</v>
+      </c>
+      <c r="K69" t="b">
+        <v>1</v>
+      </c>
+      <c r="L69" t="s">
+        <v>18</v>
+      </c>
+      <c r="M69" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>13</v>
+      </c>
+      <c r="B70" t="s">
+        <v>99</v>
+      </c>
+      <c r="C70" t="s">
+        <v>136</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F70" t="s">
+        <v>14</v>
+      </c>
+      <c r="G70" t="s">
+        <v>15</v>
+      </c>
+      <c r="H70" t="s">
+        <v>16</v>
+      </c>
+      <c r="I70" t="s">
+        <v>61</v>
+      </c>
+      <c r="J70" t="s">
+        <v>24</v>
+      </c>
+      <c r="K70" t="b">
+        <v>1</v>
+      </c>
+      <c r="L70" t="s">
+        <v>18</v>
+      </c>
+      <c r="M70" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>13</v>
+      </c>
+      <c r="B71" t="s">
+        <v>99</v>
+      </c>
+      <c r="C71" t="s">
+        <v>137</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F71" t="s">
+        <v>14</v>
+      </c>
+      <c r="G71" t="s">
+        <v>15</v>
+      </c>
+      <c r="H71" t="s">
+        <v>16</v>
+      </c>
+      <c r="I71" t="s">
+        <v>61</v>
+      </c>
+      <c r="J71" t="s">
+        <v>24</v>
+      </c>
+      <c r="K71" t="b">
+        <v>1</v>
+      </c>
+      <c r="L71" t="s">
+        <v>18</v>
+      </c>
+      <c r="M71" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>13</v>
+      </c>
+      <c r="B72" t="s">
+        <v>99</v>
+      </c>
+      <c r="C72" t="s">
+        <v>137</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F72" t="s">
+        <v>14</v>
+      </c>
+      <c r="G72" t="s">
+        <v>15</v>
+      </c>
+      <c r="H72" t="s">
+        <v>16</v>
+      </c>
+      <c r="I72" t="s">
+        <v>61</v>
+      </c>
+      <c r="J72" t="s">
+        <v>24</v>
+      </c>
+      <c r="K72" t="b">
+        <v>1</v>
+      </c>
+      <c r="L72" t="s">
+        <v>18</v>
+      </c>
+      <c r="M72" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>13</v>
+      </c>
+      <c r="B73" t="s">
+        <v>99</v>
+      </c>
+      <c r="C73" t="s">
+        <v>137</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F73" t="s">
+        <v>14</v>
+      </c>
+      <c r="G73" t="s">
+        <v>15</v>
+      </c>
+      <c r="H73" t="s">
+        <v>16</v>
+      </c>
+      <c r="I73" t="s">
+        <v>61</v>
+      </c>
+      <c r="J73" t="s">
+        <v>24</v>
+      </c>
+      <c r="K73" t="b">
+        <v>1</v>
+      </c>
+      <c r="L73" t="s">
+        <v>18</v>
+      </c>
+      <c r="M73" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>13</v>
+      </c>
+      <c r="B74" t="s">
+        <v>99</v>
+      </c>
+      <c r="C74" t="s">
+        <v>137</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F74" t="s">
+        <v>14</v>
+      </c>
+      <c r="G74" t="s">
+        <v>15</v>
+      </c>
+      <c r="H74" t="s">
+        <v>16</v>
+      </c>
+      <c r="I74" t="s">
+        <v>61</v>
+      </c>
+      <c r="J74" t="s">
+        <v>24</v>
+      </c>
+      <c r="K74" t="b">
+        <v>1</v>
+      </c>
+      <c r="L74" t="s">
+        <v>18</v>
+      </c>
+      <c r="M74" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
0.8.12 - Back to Mobile.
</commit_message>
<xml_diff>
--- a/keel_trb_smart_template.xlsx
+++ b/keel_trb_smart_template.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F695D5D-BFA6-47D9-8F5F-B1E3ECE9519A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883AF90D-6AD6-4198-A23F-B8027F3405A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="147">
   <si>
     <t>Function (Select from List)</t>
   </si>
@@ -439,6 +439,24 @@
   </si>
   <si>
     <t>Practice Position fixes by radar</t>
+  </si>
+  <si>
+    <t>Maintain a safe engineering watch</t>
+  </si>
+  <si>
+    <t>Relieve and hand over the watch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow the correct procedure for handling over a watch at sea. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow the correct procedure for handling over a watch in port. </t>
+  </si>
+  <si>
+    <t>Follow the correct procedure for taking over and accepting a watch at sea</t>
+  </si>
+  <si>
+    <t>Follow the correct procedure for taking over and accepting a watch in port</t>
   </si>
 </sst>
 </file>
@@ -491,10 +509,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -834,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -3257,7 +3274,7 @@
       <c r="C61" t="s">
         <v>125</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="D61" t="s">
         <v>127</v>
       </c>
       <c r="F61" t="s">
@@ -3295,7 +3312,7 @@
       <c r="C62" t="s">
         <v>125</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="D62" t="s">
         <v>128</v>
       </c>
       <c r="F62" t="s">
@@ -3333,7 +3350,7 @@
       <c r="C63" t="s">
         <v>125</v>
       </c>
-      <c r="D63" s="2" t="s">
+      <c r="D63" t="s">
         <v>129</v>
       </c>
       <c r="F63" t="s">
@@ -3371,7 +3388,7 @@
       <c r="C64" t="s">
         <v>125</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="D64" t="s">
         <v>130</v>
       </c>
       <c r="F64" t="s">
@@ -3409,7 +3426,7 @@
       <c r="C65" t="s">
         <v>131</v>
       </c>
-      <c r="D65" s="2" t="s">
+      <c r="D65" t="s">
         <v>132</v>
       </c>
       <c r="F65" t="s">
@@ -3447,7 +3464,7 @@
       <c r="C66" t="s">
         <v>131</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="D66" t="s">
         <v>133</v>
       </c>
       <c r="F66" t="s">
@@ -3485,7 +3502,7 @@
       <c r="C67" t="s">
         <v>131</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="D67" t="s">
         <v>134</v>
       </c>
       <c r="F67" t="s">
@@ -3523,7 +3540,7 @@
       <c r="C68" t="s">
         <v>131</v>
       </c>
-      <c r="D68" s="2" t="s">
+      <c r="D68" t="s">
         <v>135</v>
       </c>
       <c r="F68" t="s">
@@ -3561,7 +3578,7 @@
       <c r="C69" t="s">
         <v>136</v>
       </c>
-      <c r="D69" s="2" t="s">
+      <c r="D69" t="s">
         <v>123</v>
       </c>
       <c r="F69" t="s">
@@ -3599,7 +3616,7 @@
       <c r="C70" t="s">
         <v>136</v>
       </c>
-      <c r="D70" s="2" t="s">
+      <c r="D70" t="s">
         <v>114</v>
       </c>
       <c r="F70" t="s">
@@ -3637,7 +3654,7 @@
       <c r="C71" t="s">
         <v>137</v>
       </c>
-      <c r="D71" s="2" t="s">
+      <c r="D71" t="s">
         <v>138</v>
       </c>
       <c r="F71" t="s">
@@ -3675,7 +3692,7 @@
       <c r="C72" t="s">
         <v>137</v>
       </c>
-      <c r="D72" s="2" t="s">
+      <c r="D72" t="s">
         <v>139</v>
       </c>
       <c r="F72" t="s">
@@ -3713,7 +3730,7 @@
       <c r="C73" t="s">
         <v>137</v>
       </c>
-      <c r="D73" s="2" t="s">
+      <c r="D73" t="s">
         <v>140</v>
       </c>
       <c r="F73" t="s">
@@ -3751,7 +3768,7 @@
       <c r="C74" t="s">
         <v>137</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="D74" t="s">
         <v>138</v>
       </c>
       <c r="F74" t="s">
@@ -3776,6 +3793,158 @@
         <v>18</v>
       </c>
       <c r="M74" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>33</v>
+      </c>
+      <c r="B75" t="s">
+        <v>141</v>
+      </c>
+      <c r="C75" t="s">
+        <v>142</v>
+      </c>
+      <c r="D75" t="s">
+        <v>143</v>
+      </c>
+      <c r="F75" t="s">
+        <v>42</v>
+      </c>
+      <c r="G75" t="s">
+        <v>22</v>
+      </c>
+      <c r="H75" t="s">
+        <v>23</v>
+      </c>
+      <c r="I75" t="s">
+        <v>61</v>
+      </c>
+      <c r="J75" t="s">
+        <v>24</v>
+      </c>
+      <c r="K75" t="b">
+        <v>1</v>
+      </c>
+      <c r="L75" t="s">
+        <v>18</v>
+      </c>
+      <c r="M75" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>33</v>
+      </c>
+      <c r="B76" t="s">
+        <v>141</v>
+      </c>
+      <c r="C76" t="s">
+        <v>142</v>
+      </c>
+      <c r="D76" t="s">
+        <v>144</v>
+      </c>
+      <c r="F76" t="s">
+        <v>42</v>
+      </c>
+      <c r="G76" t="s">
+        <v>22</v>
+      </c>
+      <c r="H76" t="s">
+        <v>23</v>
+      </c>
+      <c r="I76" t="s">
+        <v>61</v>
+      </c>
+      <c r="J76" t="s">
+        <v>24</v>
+      </c>
+      <c r="K76" t="b">
+        <v>1</v>
+      </c>
+      <c r="L76" t="s">
+        <v>18</v>
+      </c>
+      <c r="M76" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>33</v>
+      </c>
+      <c r="B77" t="s">
+        <v>141</v>
+      </c>
+      <c r="C77" t="s">
+        <v>142</v>
+      </c>
+      <c r="D77" t="s">
+        <v>145</v>
+      </c>
+      <c r="F77" t="s">
+        <v>42</v>
+      </c>
+      <c r="G77" t="s">
+        <v>22</v>
+      </c>
+      <c r="H77" t="s">
+        <v>23</v>
+      </c>
+      <c r="I77" t="s">
+        <v>61</v>
+      </c>
+      <c r="J77" t="s">
+        <v>24</v>
+      </c>
+      <c r="K77" t="b">
+        <v>1</v>
+      </c>
+      <c r="L77" t="s">
+        <v>18</v>
+      </c>
+      <c r="M77" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>33</v>
+      </c>
+      <c r="B78" t="s">
+        <v>141</v>
+      </c>
+      <c r="C78" t="s">
+        <v>142</v>
+      </c>
+      <c r="D78" t="s">
+        <v>146</v>
+      </c>
+      <c r="F78" t="s">
+        <v>42</v>
+      </c>
+      <c r="G78" t="s">
+        <v>22</v>
+      </c>
+      <c r="H78" t="s">
+        <v>23</v>
+      </c>
+      <c r="I78" t="s">
+        <v>61</v>
+      </c>
+      <c r="J78" t="s">
+        <v>24</v>
+      </c>
+      <c r="K78" t="b">
+        <v>1</v>
+      </c>
+      <c r="L78" t="s">
+        <v>18</v>
+      </c>
+      <c r="M78" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
0.9.0 - TRB Tasks import bug resolved.
</commit_message>
<xml_diff>
--- a/keel_trb_smart_template.xlsx
+++ b/keel_trb_smart_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883AF90D-6AD6-4198-A23F-B8027F3405A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7B2821-D06A-4F1A-81E0-5ADE633A402F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,9 +18,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="147">
   <si>
-    <t>Function (Select from List)</t>
-  </si>
-  <si>
     <t>Section / Topic</t>
   </si>
   <si>
@@ -457,6 +454,9 @@
   </si>
   <si>
     <t>Follow the correct procedure for taking over and accepting a watch in port</t>
+  </si>
+  <si>
+    <t>Function</t>
   </si>
 </sst>
 </file>
@@ -869,3083 +869,3083 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" t="s">
         <v>57</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>58</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>59</v>
       </c>
-      <c r="E2" t="s">
-        <v>60</v>
-      </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K2" t="b">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
         <v>57</v>
       </c>
-      <c r="C3" t="s">
-        <v>58</v>
-      </c>
       <c r="D3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K3" t="b">
         <v>1</v>
       </c>
       <c r="L3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" t="s">
         <v>57</v>
       </c>
-      <c r="C4" t="s">
-        <v>58</v>
-      </c>
       <c r="D4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K4" t="b">
         <v>1</v>
       </c>
       <c r="L4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" t="s">
         <v>57</v>
       </c>
-      <c r="C5" t="s">
-        <v>58</v>
-      </c>
       <c r="D5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K5" t="b">
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
         <v>57</v>
       </c>
-      <c r="C6" t="s">
-        <v>58</v>
-      </c>
       <c r="D6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K6" t="b">
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" t="s">
         <v>57</v>
       </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
       <c r="D7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K7" t="b">
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" t="s">
         <v>57</v>
       </c>
-      <c r="C8" t="s">
-        <v>58</v>
-      </c>
       <c r="D8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K8" t="b">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s">
         <v>57</v>
       </c>
-      <c r="C9" t="s">
-        <v>58</v>
-      </c>
       <c r="D9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K9" t="b">
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
         <v>57</v>
       </c>
-      <c r="C10" t="s">
-        <v>58</v>
-      </c>
       <c r="D10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K10" t="b">
         <v>1</v>
       </c>
       <c r="L10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" t="s">
         <v>57</v>
       </c>
-      <c r="C11" t="s">
-        <v>58</v>
-      </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K11" t="b">
         <v>1</v>
       </c>
       <c r="L11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" t="s">
         <v>57</v>
       </c>
-      <c r="C12" t="s">
-        <v>58</v>
-      </c>
       <c r="D12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K12" t="b">
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
         <v>57</v>
       </c>
-      <c r="C13" t="s">
-        <v>58</v>
-      </c>
       <c r="D13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K13" t="b">
         <v>1</v>
       </c>
       <c r="L13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
         <v>57</v>
       </c>
-      <c r="C14" t="s">
-        <v>58</v>
-      </c>
       <c r="D14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K14" t="b">
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" t="s">
         <v>57</v>
       </c>
-      <c r="C15" t="s">
-        <v>58</v>
-      </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K15" t="b">
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" t="s">
         <v>57</v>
       </c>
-      <c r="C16" t="s">
-        <v>58</v>
-      </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K16" t="b">
         <v>1</v>
       </c>
       <c r="L16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
         <v>57</v>
       </c>
-      <c r="C17" t="s">
-        <v>58</v>
-      </c>
       <c r="D17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K17" t="b">
         <v>1</v>
       </c>
       <c r="L17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" t="s">
         <v>57</v>
       </c>
-      <c r="C18" t="s">
-        <v>58</v>
-      </c>
       <c r="D18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K18" t="b">
         <v>1</v>
       </c>
       <c r="L18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" t="s">
         <v>57</v>
       </c>
-      <c r="C19" t="s">
-        <v>58</v>
-      </c>
       <c r="D19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K19" t="b">
         <v>1</v>
       </c>
       <c r="L19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" t="s">
         <v>57</v>
       </c>
-      <c r="C20" t="s">
-        <v>58</v>
-      </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K20" t="b">
         <v>1</v>
       </c>
       <c r="L20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" t="s">
         <v>57</v>
       </c>
-      <c r="C21" t="s">
-        <v>58</v>
-      </c>
       <c r="D21" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K21" t="b">
         <v>1</v>
       </c>
       <c r="L21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" t="s">
         <v>57</v>
       </c>
-      <c r="C22" t="s">
-        <v>58</v>
-      </c>
       <c r="D22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K22" t="b">
         <v>1</v>
       </c>
       <c r="L22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" t="s">
         <v>57</v>
       </c>
-      <c r="C23" t="s">
-        <v>58</v>
-      </c>
       <c r="D23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K23" t="b">
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" t="s">
         <v>57</v>
       </c>
-      <c r="C24" t="s">
-        <v>58</v>
-      </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K24" t="b">
         <v>1</v>
       </c>
       <c r="L24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" t="s">
         <v>57</v>
       </c>
-      <c r="C25" t="s">
-        <v>58</v>
-      </c>
       <c r="D25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K25" t="b">
         <v>1</v>
       </c>
       <c r="L25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" t="s">
         <v>57</v>
       </c>
-      <c r="C26" t="s">
-        <v>58</v>
-      </c>
       <c r="D26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K26" t="b">
         <v>1</v>
       </c>
       <c r="L26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" t="s">
         <v>57</v>
       </c>
-      <c r="C27" t="s">
-        <v>58</v>
-      </c>
       <c r="D27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K27" t="b">
         <v>1</v>
       </c>
       <c r="L27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M27" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" t="s">
         <v>57</v>
       </c>
-      <c r="C28" t="s">
-        <v>58</v>
-      </c>
       <c r="D28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G28" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K28" t="b">
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" t="s">
         <v>57</v>
       </c>
-      <c r="C29" t="s">
-        <v>58</v>
-      </c>
       <c r="D29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K29" t="b">
         <v>1</v>
       </c>
       <c r="L29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" t="s">
         <v>57</v>
       </c>
-      <c r="C30" t="s">
-        <v>58</v>
-      </c>
       <c r="D30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H30" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J30" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K30" t="b">
         <v>1</v>
       </c>
       <c r="L30" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" t="s">
         <v>57</v>
       </c>
-      <c r="C31" t="s">
-        <v>58</v>
-      </c>
       <c r="D31" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H31" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I31" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K31" t="b">
         <v>1</v>
       </c>
       <c r="L31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B32" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" t="s">
         <v>57</v>
       </c>
-      <c r="C32" t="s">
-        <v>58</v>
-      </c>
       <c r="D32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I32" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K32" t="b">
         <v>1</v>
       </c>
       <c r="L32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" t="s">
         <v>57</v>
       </c>
-      <c r="C33" t="s">
-        <v>58</v>
-      </c>
       <c r="D33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E33" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H33" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I33" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J33" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K33" t="b">
         <v>1</v>
       </c>
       <c r="L33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M33" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" t="s">
         <v>57</v>
       </c>
-      <c r="C34" t="s">
-        <v>58</v>
-      </c>
       <c r="D34" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E34" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H34" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I34" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J34" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K34" t="b">
         <v>1</v>
       </c>
       <c r="L34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M34" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B35" t="s">
+        <v>56</v>
+      </c>
+      <c r="C35" t="s">
         <v>57</v>
       </c>
-      <c r="C35" t="s">
-        <v>58</v>
-      </c>
       <c r="D35" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G35" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H35" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I35" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K35" t="b">
         <v>1</v>
       </c>
       <c r="L35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
+        <v>56</v>
+      </c>
+      <c r="C36" t="s">
         <v>57</v>
       </c>
-      <c r="C36" t="s">
-        <v>58</v>
-      </c>
       <c r="D36" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E36" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G36" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H36" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J36" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K36" t="b">
         <v>1</v>
       </c>
       <c r="L36" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
+        <v>56</v>
+      </c>
+      <c r="C37" t="s">
         <v>57</v>
       </c>
-      <c r="C37" t="s">
-        <v>58</v>
-      </c>
       <c r="D37" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F37" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G37" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H37" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K37" t="b">
         <v>1</v>
       </c>
       <c r="L37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B38" t="s">
+        <v>56</v>
+      </c>
+      <c r="C38" t="s">
         <v>57</v>
       </c>
-      <c r="C38" t="s">
-        <v>58</v>
-      </c>
       <c r="D38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G38" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H38" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K38" t="b">
         <v>1</v>
       </c>
       <c r="L38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B39" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" t="s">
         <v>57</v>
       </c>
-      <c r="C39" t="s">
-        <v>58</v>
-      </c>
       <c r="D39" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E39" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F39" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G39" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H39" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K39" t="b">
         <v>1</v>
       </c>
       <c r="L39" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M39" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B40" t="s">
+        <v>98</v>
+      </c>
+      <c r="C40" t="s">
         <v>99</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>100</v>
       </c>
-      <c r="D40" t="s">
-        <v>101</v>
-      </c>
       <c r="F40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G40" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H40" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J40" t="s">
+        <v>23</v>
+      </c>
+      <c r="K40" t="b">
+        <v>1</v>
+      </c>
+      <c r="L40" t="s">
         <v>24</v>
       </c>
-      <c r="K40" t="b">
-        <v>1</v>
-      </c>
-      <c r="L40" t="s">
-        <v>25</v>
-      </c>
       <c r="M40" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" t="s">
+        <v>98</v>
+      </c>
+      <c r="C41" t="s">
         <v>99</v>
       </c>
-      <c r="C41" t="s">
-        <v>100</v>
-      </c>
       <c r="D41" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F41" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H41" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J41" t="s">
+        <v>23</v>
+      </c>
+      <c r="K41" t="b">
+        <v>1</v>
+      </c>
+      <c r="L41" t="s">
         <v>24</v>
       </c>
-      <c r="K41" t="b">
-        <v>1</v>
-      </c>
-      <c r="L41" t="s">
-        <v>25</v>
-      </c>
       <c r="M41" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B42" t="s">
+        <v>98</v>
+      </c>
+      <c r="C42" t="s">
         <v>99</v>
       </c>
-      <c r="C42" t="s">
-        <v>100</v>
-      </c>
       <c r="D42" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H42" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I42" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J42" t="s">
+        <v>23</v>
+      </c>
+      <c r="K42" t="b">
+        <v>1</v>
+      </c>
+      <c r="L42" t="s">
         <v>24</v>
       </c>
-      <c r="K42" t="b">
-        <v>1</v>
-      </c>
-      <c r="L42" t="s">
-        <v>25</v>
-      </c>
       <c r="M42" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B43" t="s">
+        <v>98</v>
+      </c>
+      <c r="C43" t="s">
         <v>99</v>
       </c>
-      <c r="C43" t="s">
-        <v>100</v>
-      </c>
       <c r="D43" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F43" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I43" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J43" t="s">
+        <v>23</v>
+      </c>
+      <c r="K43" t="b">
+        <v>1</v>
+      </c>
+      <c r="L43" t="s">
         <v>24</v>
       </c>
-      <c r="K43" t="b">
-        <v>1</v>
-      </c>
-      <c r="L43" t="s">
-        <v>25</v>
-      </c>
       <c r="M43" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B44" t="s">
+        <v>98</v>
+      </c>
+      <c r="C44" t="s">
         <v>99</v>
       </c>
-      <c r="C44" t="s">
-        <v>100</v>
-      </c>
       <c r="D44" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F44" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G44" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H44" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J44" t="s">
+        <v>23</v>
+      </c>
+      <c r="K44" t="b">
+        <v>1</v>
+      </c>
+      <c r="L44" t="s">
         <v>24</v>
       </c>
-      <c r="K44" t="b">
-        <v>1</v>
-      </c>
-      <c r="L44" t="s">
-        <v>25</v>
-      </c>
       <c r="M44" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B45" t="s">
+        <v>98</v>
+      </c>
+      <c r="C45" t="s">
         <v>99</v>
       </c>
-      <c r="C45" t="s">
-        <v>100</v>
-      </c>
       <c r="D45" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F45" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G45" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H45" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I45" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J45" t="s">
+        <v>23</v>
+      </c>
+      <c r="K45" t="b">
+        <v>1</v>
+      </c>
+      <c r="L45" t="s">
         <v>24</v>
       </c>
-      <c r="K45" t="b">
-        <v>1</v>
-      </c>
-      <c r="L45" t="s">
-        <v>25</v>
-      </c>
       <c r="M45" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B46" t="s">
+        <v>98</v>
+      </c>
+      <c r="C46" t="s">
         <v>99</v>
       </c>
-      <c r="C46" t="s">
-        <v>100</v>
-      </c>
       <c r="D46" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G46" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H46" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I46" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J46" t="s">
+        <v>23</v>
+      </c>
+      <c r="K46" t="b">
+        <v>1</v>
+      </c>
+      <c r="L46" t="s">
         <v>24</v>
       </c>
-      <c r="K46" t="b">
-        <v>1</v>
-      </c>
-      <c r="L46" t="s">
-        <v>25</v>
-      </c>
       <c r="M46" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B47" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C47" t="s">
+        <v>107</v>
+      </c>
+      <c r="D47" t="s">
         <v>108</v>
       </c>
-      <c r="D47" t="s">
-        <v>109</v>
-      </c>
       <c r="F47" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G47" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H47" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I47" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K47" t="b">
         <v>1</v>
       </c>
       <c r="L47" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M47" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C48" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D48" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H48" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I48" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J48" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K48" t="b">
         <v>1</v>
       </c>
       <c r="L48" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M48" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B49" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D49" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F49" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I49" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K49" t="b">
         <v>1</v>
       </c>
       <c r="L49" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M49" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B50" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C50" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D50" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H50" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I50" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J50" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K50" t="b">
         <v>1</v>
       </c>
       <c r="L50" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M50" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B51" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D51" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F51" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G51" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H51" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I51" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J51" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K51" t="b">
         <v>1</v>
       </c>
       <c r="L51" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M51" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C52" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D52" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F52" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G52" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H52" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I52" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J52" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K52" t="b">
         <v>1</v>
       </c>
       <c r="L52" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M52" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C53" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D53" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F53" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G53" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H53" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I53" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J53" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K53" t="b">
         <v>1</v>
       </c>
       <c r="L53" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M53" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C54" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D54" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H54" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I54" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J54" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K54" t="b">
         <v>1</v>
       </c>
       <c r="L54" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M54" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B55" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C55" t="s">
+        <v>115</v>
+      </c>
+      <c r="D55" t="s">
         <v>116</v>
       </c>
-      <c r="D55" t="s">
-        <v>117</v>
-      </c>
       <c r="F55" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H55" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J55" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K55" t="b">
         <v>1</v>
       </c>
       <c r="L55" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M55" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C56" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D56" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I56" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J56" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K56" t="b">
         <v>1</v>
       </c>
       <c r="L56" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M56" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C57" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F57" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G57" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H57" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I57" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J57" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K57" t="b">
         <v>1</v>
       </c>
       <c r="L57" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M57" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C58" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D58" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G58" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H58" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I58" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J58" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K58" t="b">
         <v>1</v>
       </c>
       <c r="L58" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M58" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D59" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G59" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H59" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I59" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J59" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K59" t="b">
         <v>1</v>
       </c>
       <c r="L59" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M59" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B60" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C60" t="s">
+        <v>124</v>
+      </c>
+      <c r="D60" t="s">
         <v>125</v>
       </c>
-      <c r="D60" t="s">
-        <v>126</v>
-      </c>
       <c r="F60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G60" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H60" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I60" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J60" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K60" t="b">
         <v>1</v>
       </c>
       <c r="L60" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M60" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C61" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D61" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F61" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G61" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H61" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J61" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K61" t="b">
         <v>1</v>
       </c>
       <c r="L61" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M61" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B62" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C62" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D62" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F62" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G62" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H62" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J62" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K62" t="b">
         <v>1</v>
       </c>
       <c r="L62" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M62" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B63" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C63" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D63" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G63" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H63" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I63" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J63" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K63" t="b">
         <v>1</v>
       </c>
       <c r="L63" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B64" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C64" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D64" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G64" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H64" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I64" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J64" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K64" t="b">
         <v>1</v>
       </c>
       <c r="L64" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M64" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C65" t="s">
+        <v>130</v>
+      </c>
+      <c r="D65" t="s">
         <v>131</v>
       </c>
-      <c r="D65" t="s">
-        <v>132</v>
-      </c>
       <c r="F65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G65" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H65" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I65" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J65" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K65" t="b">
         <v>1</v>
       </c>
       <c r="L65" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M65" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B66" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C66" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D66" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G66" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H66" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I66" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J66" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K66" t="b">
         <v>1</v>
       </c>
       <c r="L66" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M66" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B67" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C67" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D67" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H67" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I67" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J67" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K67" t="b">
         <v>1</v>
       </c>
       <c r="L67" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M67" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B68" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C68" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D68" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F68" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G68" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H68" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I68" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J68" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K68" t="b">
         <v>1</v>
       </c>
       <c r="L68" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M68" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B69" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C69" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D69" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F69" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G69" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H69" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I69" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J69" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K69" t="b">
         <v>1</v>
       </c>
       <c r="L69" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M69" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B70" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C70" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D70" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F70" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G70" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H70" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I70" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J70" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K70" t="b">
         <v>1</v>
       </c>
       <c r="L70" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M70" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B71" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C71" t="s">
+        <v>136</v>
+      </c>
+      <c r="D71" t="s">
         <v>137</v>
       </c>
-      <c r="D71" t="s">
-        <v>138</v>
-      </c>
       <c r="F71" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G71" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H71" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I71" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J71" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K71" t="b">
         <v>1</v>
       </c>
       <c r="L71" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M71" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B72" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C72" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D72" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H72" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I72" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J72" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K72" t="b">
         <v>1</v>
       </c>
       <c r="L72" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M72" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B73" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C73" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D73" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F73" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G73" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H73" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I73" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J73" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K73" t="b">
         <v>1</v>
       </c>
       <c r="L73" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M73" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B74" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C74" t="s">
+        <v>136</v>
+      </c>
+      <c r="D74" t="s">
         <v>137</v>
       </c>
-      <c r="D74" t="s">
-        <v>138</v>
-      </c>
       <c r="F74" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G74" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H74" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I74" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J74" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K74" t="b">
         <v>1</v>
       </c>
       <c r="L74" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M74" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B75" t="s">
+        <v>140</v>
+      </c>
+      <c r="C75" t="s">
         <v>141</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>142</v>
       </c>
-      <c r="D75" t="s">
-        <v>143</v>
-      </c>
       <c r="F75" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G75" t="s">
+        <v>21</v>
+      </c>
+      <c r="H75" t="s">
         <v>22</v>
       </c>
-      <c r="H75" t="s">
-        <v>23</v>
-      </c>
       <c r="I75" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J75" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K75" t="b">
         <v>1</v>
       </c>
       <c r="L75" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M75" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B76" t="s">
+        <v>140</v>
+      </c>
+      <c r="C76" t="s">
         <v>141</v>
       </c>
-      <c r="C76" t="s">
-        <v>142</v>
-      </c>
       <c r="D76" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F76" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G76" t="s">
+        <v>21</v>
+      </c>
+      <c r="H76" t="s">
         <v>22</v>
       </c>
-      <c r="H76" t="s">
-        <v>23</v>
-      </c>
       <c r="I76" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J76" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K76" t="b">
         <v>1</v>
       </c>
       <c r="L76" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M76" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B77" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" t="s">
         <v>141</v>
       </c>
-      <c r="C77" t="s">
-        <v>142</v>
-      </c>
       <c r="D77" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F77" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G77" t="s">
+        <v>21</v>
+      </c>
+      <c r="H77" t="s">
         <v>22</v>
       </c>
-      <c r="H77" t="s">
-        <v>23</v>
-      </c>
       <c r="I77" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J77" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K77" t="b">
         <v>1</v>
       </c>
       <c r="L77" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M77" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B78" t="s">
+        <v>140</v>
+      </c>
+      <c r="C78" t="s">
         <v>141</v>
       </c>
-      <c r="C78" t="s">
-        <v>142</v>
-      </c>
       <c r="D78" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F78" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G78" t="s">
+        <v>21</v>
+      </c>
+      <c r="H78" t="s">
         <v>22</v>
       </c>
-      <c r="H78" t="s">
-        <v>23</v>
-      </c>
       <c r="I78" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J78" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K78" t="b">
         <v>1</v>
       </c>
       <c r="L78" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M78" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -4015,168 +4015,168 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" t="s">
-        <v>17</v>
-      </c>
       <c r="F1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" t="s">
         <v>18</v>
-      </c>
-      <c r="G1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>21</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>22</v>
       </c>
-      <c r="D2" t="s">
-        <v>23</v>
-      </c>
       <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
         <v>24</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>25</v>
-      </c>
-      <c r="G2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>28</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>29</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>30</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>31</v>
-      </c>
-      <c r="G3" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>35</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>36</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
         <v>38</v>
       </c>
-      <c r="B5" t="s">
+      <c r="E5" t="s">
         <v>39</v>
-      </c>
-      <c r="E5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
         <v>41</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
         <v>42</v>
-      </c>
-      <c r="E6" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" t="s">
+      <c r="E7" t="s">
         <v>45</v>
-      </c>
-      <c r="E7" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>